<commit_message>
Add Master Data Tracking and new SAP item requests with duplicate checks.
Give requesters a single page to find an item, block duplicates, follow request progress, and receive a created-in-SAP notice, while keeping studio and pipeline tooling for master-data staff.
</commit_message>
<xml_diff>
--- a/assets/templates/SAP Item Template column Mapping data 2.xlsx
+++ b/assets/templates/SAP Item Template column Mapping data 2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/som_home/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Som_SSD_T7/Workspace/Kiswok_Internal_on_AI/assets/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D0D098-F789-BA46-B873-4F461DCB3A67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A97E4DD-BA63-A545-9876-457220D84970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="38400" windowHeight="22880" xr2:uid="{89531264-3F51-174A-B534-72D158616AFA}"/>
   </bookViews>
@@ -16,10 +16,7 @@
     <sheet name="Template Mapping " sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId3"/>
-  </externalReferences>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" refMode="R1C1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="169">
   <si>
     <t>Default Fixed value</t>
   </si>
@@ -536,6 +533,18 @@
   </si>
   <si>
     <t>Table available</t>
+  </si>
+  <si>
+    <t>Consumable</t>
+  </si>
+  <si>
+    <t>DRILL BIT 10MM X 116 FLUTE LENGTH (T/S)</t>
+  </si>
+  <si>
+    <t>EN</t>
+  </si>
+  <si>
+    <t>EA</t>
   </si>
 </sst>
 </file>
@@ -719,16 +728,16 @@
     <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -746,585 +755,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId3"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Item Master Consolidated"/>
-      <sheetName val="Single Row template"/>
-      <sheetName val="Raw data"/>
-      <sheetName val="Sheet3"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2">
-        <row r="1">
-          <cell r="A1" t="str">
-            <v>RAWMATCODE</v>
-          </cell>
-          <cell r="B1" t="str">
-            <v>Product Type</v>
-          </cell>
-          <cell r="C1" t="str">
-            <v>grntype</v>
-          </cell>
-          <cell r="D1" t="str">
-            <v>Product Group</v>
-          </cell>
-          <cell r="E1" t="str">
-            <v>Rawmatname</v>
-          </cell>
-          <cell r="F1" t="str">
-            <v>lang</v>
-          </cell>
-          <cell r="G1" t="str">
-            <v>baseuom</v>
-          </cell>
-          <cell r="H1" t="str">
-            <v>PurchaseUom</v>
-          </cell>
-          <cell r="I1" t="str">
-            <v>LONG TEXT</v>
-          </cell>
-          <cell r="J1" t="str">
-            <v>WeightUom</v>
-          </cell>
-          <cell r="K1" t="str">
-            <v>Weight</v>
-          </cell>
-          <cell r="L1" t="str">
-            <v>hsncode</v>
-          </cell>
-          <cell r="M1" t="str">
-            <v>LocationID</v>
-          </cell>
-          <cell r="N1" t="str">
-            <v>sap_plantcode</v>
-          </cell>
-          <cell r="O1" t="str">
-            <v>storage_location</v>
-          </cell>
-          <cell r="P1" t="str">
-            <v>GrnTypeId</v>
-          </cell>
-          <cell r="Q1" t="str">
-            <v>RawMatID</v>
-          </cell>
-          <cell r="R1" t="str">
-            <v>profitcentercode</v>
-          </cell>
-        </row>
-        <row r="2">
-          <cell r="A2" t="str">
-            <v>CONGEDB0032</v>
-          </cell>
-          <cell r="B2" t="str">
-            <v>ZRAW</v>
-          </cell>
-          <cell r="C2" t="str">
-            <v>Consumable</v>
-          </cell>
-          <cell r="D2" t="str">
-            <v>NULL</v>
-          </cell>
-          <cell r="E2" t="str">
-            <v>DRILL BIT 10MM X 116 FLUTE LENGTH (T/S)</v>
-          </cell>
-          <cell r="F2" t="str">
-            <v>EN</v>
-          </cell>
-          <cell r="G2" t="str">
-            <v>EA</v>
-          </cell>
-          <cell r="H2" t="str">
-            <v>EA</v>
-          </cell>
-          <cell r="K2">
-            <v>0</v>
-          </cell>
-          <cell r="L2">
-            <v>82070000</v>
-          </cell>
-          <cell r="M2">
-            <v>5</v>
-          </cell>
-          <cell r="N2">
-            <v>2004</v>
-          </cell>
-          <cell r="O2" t="str">
-            <v>CNCD</v>
-          </cell>
-          <cell r="P2">
-            <v>2</v>
-          </cell>
-          <cell r="Q2">
-            <v>394649</v>
-          </cell>
-          <cell r="R2">
-            <v>200401</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="A3" t="str">
-            <v>CONGEDB0032</v>
-          </cell>
-          <cell r="B3" t="str">
-            <v>ZRAW</v>
-          </cell>
-          <cell r="C3" t="str">
-            <v>Consumable</v>
-          </cell>
-          <cell r="D3" t="str">
-            <v>NULL</v>
-          </cell>
-          <cell r="E3" t="str">
-            <v>DRILL BIT 10MM X 116 FLUTE LENGTH (T/S)</v>
-          </cell>
-          <cell r="F3" t="str">
-            <v>EN</v>
-          </cell>
-          <cell r="G3" t="str">
-            <v>EA</v>
-          </cell>
-          <cell r="H3" t="str">
-            <v>EA</v>
-          </cell>
-          <cell r="K3">
-            <v>0</v>
-          </cell>
-          <cell r="L3">
-            <v>82070000</v>
-          </cell>
-          <cell r="M3">
-            <v>3</v>
-          </cell>
-          <cell r="N3">
-            <v>2001</v>
-          </cell>
-          <cell r="O3" t="str">
-            <v>MXST</v>
-          </cell>
-          <cell r="P3">
-            <v>2</v>
-          </cell>
-          <cell r="Q3">
-            <v>394649</v>
-          </cell>
-          <cell r="R3">
-            <v>200101</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4" t="str">
-            <v>CONGEDB0032</v>
-          </cell>
-          <cell r="B4" t="str">
-            <v>ZRAW</v>
-          </cell>
-          <cell r="C4" t="str">
-            <v>Consumable</v>
-          </cell>
-          <cell r="D4" t="str">
-            <v>NULL</v>
-          </cell>
-          <cell r="E4" t="str">
-            <v>DRILL BIT 10MM X 116 FLUTE LENGTH (T/S)</v>
-          </cell>
-          <cell r="F4" t="str">
-            <v>EN</v>
-          </cell>
-          <cell r="G4" t="str">
-            <v>EA</v>
-          </cell>
-          <cell r="H4" t="str">
-            <v>EA</v>
-          </cell>
-          <cell r="K4">
-            <v>0</v>
-          </cell>
-          <cell r="L4">
-            <v>82070000</v>
-          </cell>
-          <cell r="M4">
-            <v>3</v>
-          </cell>
-          <cell r="N4">
-            <v>2001</v>
-          </cell>
-          <cell r="O4" t="str">
-            <v>SUBC</v>
-          </cell>
-          <cell r="P4">
-            <v>2</v>
-          </cell>
-          <cell r="Q4">
-            <v>394649</v>
-          </cell>
-          <cell r="R4">
-            <v>200101</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5" t="str">
-            <v>CONGEDB0032</v>
-          </cell>
-          <cell r="B5" t="str">
-            <v>ZRAW</v>
-          </cell>
-          <cell r="C5" t="str">
-            <v>Consumable</v>
-          </cell>
-          <cell r="D5" t="str">
-            <v>NULL</v>
-          </cell>
-          <cell r="E5" t="str">
-            <v>DRILL BIT 10MM X 116 FLUTE LENGTH (T/S)</v>
-          </cell>
-          <cell r="F5" t="str">
-            <v>EN</v>
-          </cell>
-          <cell r="G5" t="str">
-            <v>EA</v>
-          </cell>
-          <cell r="H5" t="str">
-            <v>EA</v>
-          </cell>
-          <cell r="K5">
-            <v>0</v>
-          </cell>
-          <cell r="L5">
-            <v>82070000</v>
-          </cell>
-          <cell r="M5">
-            <v>2</v>
-          </cell>
-          <cell r="N5">
-            <v>2002</v>
-          </cell>
-          <cell r="O5" t="str">
-            <v>VNRT</v>
-          </cell>
-          <cell r="P5">
-            <v>2</v>
-          </cell>
-          <cell r="Q5">
-            <v>394649</v>
-          </cell>
-          <cell r="R5">
-            <v>200201</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6" t="str">
-            <v>CONGEDB0032</v>
-          </cell>
-          <cell r="B6" t="str">
-            <v>ZRAW</v>
-          </cell>
-          <cell r="C6" t="str">
-            <v>Consumable</v>
-          </cell>
-          <cell r="D6" t="str">
-            <v>NULL</v>
-          </cell>
-          <cell r="E6" t="str">
-            <v>DRILL BIT 10MM X 116 FLUTE LENGTH (T/S)</v>
-          </cell>
-          <cell r="F6" t="str">
-            <v>EN</v>
-          </cell>
-          <cell r="G6" t="str">
-            <v>EA</v>
-          </cell>
-          <cell r="H6" t="str">
-            <v>EA</v>
-          </cell>
-          <cell r="K6">
-            <v>0</v>
-          </cell>
-          <cell r="L6">
-            <v>82070000</v>
-          </cell>
-          <cell r="M6">
-            <v>2</v>
-          </cell>
-          <cell r="N6">
-            <v>2002</v>
-          </cell>
-          <cell r="O6" t="str">
-            <v>CSHT</v>
-          </cell>
-          <cell r="P6">
-            <v>2</v>
-          </cell>
-          <cell r="Q6">
-            <v>394649</v>
-          </cell>
-          <cell r="R6">
-            <v>200201</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7" t="str">
-            <v>CONGEDB0032</v>
-          </cell>
-          <cell r="B7" t="str">
-            <v>ZRAW</v>
-          </cell>
-          <cell r="C7" t="str">
-            <v>Consumable</v>
-          </cell>
-          <cell r="D7" t="str">
-            <v>NULL</v>
-          </cell>
-          <cell r="E7" t="str">
-            <v>DRILL BIT 10MM X 116 FLUTE LENGTH (T/S)</v>
-          </cell>
-          <cell r="F7" t="str">
-            <v>EN</v>
-          </cell>
-          <cell r="G7" t="str">
-            <v>EA</v>
-          </cell>
-          <cell r="H7" t="str">
-            <v>EA</v>
-          </cell>
-          <cell r="K7">
-            <v>0</v>
-          </cell>
-          <cell r="L7">
-            <v>82070000</v>
-          </cell>
-          <cell r="M7">
-            <v>3</v>
-          </cell>
-          <cell r="N7">
-            <v>2001</v>
-          </cell>
-          <cell r="O7" t="str">
-            <v>SH01</v>
-          </cell>
-          <cell r="P7">
-            <v>2</v>
-          </cell>
-          <cell r="Q7">
-            <v>394649</v>
-          </cell>
-          <cell r="R7">
-            <v>200101</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8" t="str">
-            <v>CONGEDB0032</v>
-          </cell>
-          <cell r="B8" t="str">
-            <v>ZRAW</v>
-          </cell>
-          <cell r="C8" t="str">
-            <v>Consumable</v>
-          </cell>
-          <cell r="D8" t="str">
-            <v>NULL</v>
-          </cell>
-          <cell r="E8" t="str">
-            <v>DRILL BIT 10MM X 116 FLUTE LENGTH (T/S)</v>
-          </cell>
-          <cell r="F8" t="str">
-            <v>EN</v>
-          </cell>
-          <cell r="G8" t="str">
-            <v>EA</v>
-          </cell>
-          <cell r="H8" t="str">
-            <v>EA</v>
-          </cell>
-          <cell r="K8">
-            <v>0</v>
-          </cell>
-          <cell r="L8">
-            <v>82070000</v>
-          </cell>
-          <cell r="M8">
-            <v>2</v>
-          </cell>
-          <cell r="N8">
-            <v>2002</v>
-          </cell>
-          <cell r="O8" t="str">
-            <v>JOLT</v>
-          </cell>
-          <cell r="P8">
-            <v>2</v>
-          </cell>
-          <cell r="Q8">
-            <v>394649</v>
-          </cell>
-          <cell r="R8">
-            <v>200201</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9" t="str">
-            <v>CONGEDB0032</v>
-          </cell>
-          <cell r="B9" t="str">
-            <v>ZRAW</v>
-          </cell>
-          <cell r="C9" t="str">
-            <v>Consumable</v>
-          </cell>
-          <cell r="D9" t="str">
-            <v>NULL</v>
-          </cell>
-          <cell r="E9" t="str">
-            <v>DRILL BIT 10MM X 116 FLUTE LENGTH (T/S)</v>
-          </cell>
-          <cell r="F9" t="str">
-            <v>EN</v>
-          </cell>
-          <cell r="G9" t="str">
-            <v>EA</v>
-          </cell>
-          <cell r="H9" t="str">
-            <v>EA</v>
-          </cell>
-          <cell r="K9">
-            <v>0</v>
-          </cell>
-          <cell r="L9">
-            <v>82070000</v>
-          </cell>
-          <cell r="M9">
-            <v>2</v>
-          </cell>
-          <cell r="N9">
-            <v>2002</v>
-          </cell>
-          <cell r="O9" t="str">
-            <v>MXST</v>
-          </cell>
-          <cell r="P9">
-            <v>2</v>
-          </cell>
-          <cell r="Q9">
-            <v>394649</v>
-          </cell>
-          <cell r="R9">
-            <v>200201</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10" t="str">
-            <v>CONGEDB0032</v>
-          </cell>
-          <cell r="B10" t="str">
-            <v>ZRAW</v>
-          </cell>
-          <cell r="C10" t="str">
-            <v>Consumable</v>
-          </cell>
-          <cell r="D10" t="str">
-            <v>NULL</v>
-          </cell>
-          <cell r="E10" t="str">
-            <v>DRILL BIT 10MM X 116 FLUTE LENGTH (T/S)</v>
-          </cell>
-          <cell r="F10" t="str">
-            <v>EN</v>
-          </cell>
-          <cell r="G10" t="str">
-            <v>EA</v>
-          </cell>
-          <cell r="H10" t="str">
-            <v>EA</v>
-          </cell>
-          <cell r="K10">
-            <v>0</v>
-          </cell>
-          <cell r="L10">
-            <v>82070000</v>
-          </cell>
-          <cell r="M10">
-            <v>3</v>
-          </cell>
-          <cell r="N10">
-            <v>2001</v>
-          </cell>
-          <cell r="O10" t="str">
-            <v>RGOL</v>
-          </cell>
-          <cell r="P10">
-            <v>2</v>
-          </cell>
-          <cell r="Q10">
-            <v>394649</v>
-          </cell>
-          <cell r="R10">
-            <v>200101</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11" t="str">
-            <v>CONGEDB0032</v>
-          </cell>
-          <cell r="B11" t="str">
-            <v>ZRAW</v>
-          </cell>
-          <cell r="C11" t="str">
-            <v>Consumable</v>
-          </cell>
-          <cell r="D11" t="str">
-            <v>NULL</v>
-          </cell>
-          <cell r="E11" t="str">
-            <v>DRILL BIT 10MM X 116 FLUTE LENGTH (T/S)</v>
-          </cell>
-          <cell r="F11" t="str">
-            <v>EN</v>
-          </cell>
-          <cell r="G11" t="str">
-            <v>EA</v>
-          </cell>
-          <cell r="H11" t="str">
-            <v>EA</v>
-          </cell>
-          <cell r="K11">
-            <v>0</v>
-          </cell>
-          <cell r="L11">
-            <v>82070000</v>
-          </cell>
-          <cell r="M11">
-            <v>3</v>
-          </cell>
-          <cell r="N11">
-            <v>2001</v>
-          </cell>
-          <cell r="O11" t="str">
-            <v>VNRT</v>
-          </cell>
-          <cell r="P11">
-            <v>2</v>
-          </cell>
-          <cell r="Q11">
-            <v>394649</v>
-          </cell>
-          <cell r="R11">
-            <v>200101</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="3"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1650,7 +1080,7 @@
     <col min="1" max="1" width="28.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="44.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="4" max="4" width="21.33203125" customWidth="1"/>
     <col min="5" max="5" width="36.6640625" customWidth="1"/>
     <col min="6" max="6" width="32.5" customWidth="1"/>
     <col min="7" max="7" width="28.6640625" customWidth="1"/>
@@ -1677,7 +1107,7 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="12" t="s">
         <v>115</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -1691,8 +1121,8 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="11"/>
-      <c r="B3" s="12" t="s">
+      <c r="A3" s="13"/>
+      <c r="B3" s="14" t="s">
         <v>113</v>
       </c>
       <c r="C3" s="1" t="s">
@@ -1707,61 +1137,57 @@
       <c r="F3" t="s">
         <v>127</v>
       </c>
-      <c r="G3" s="13" t="s">
+      <c r="G3" s="10" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="11"/>
-      <c r="B4" s="11"/>
+      <c r="A4" s="13"/>
+      <c r="B4" s="13"/>
       <c r="C4" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="D4" t="str">
-        <f>VLOOKUP(D2,'[1]Raw data'!1:3,3,0)</f>
-        <v>Consumable</v>
+      <c r="D4" t="s">
+        <v>165</v>
       </c>
       <c r="E4" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="11"/>
-      <c r="B5" s="11"/>
+      <c r="A5" s="13"/>
+      <c r="B5" s="13"/>
       <c r="C5" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D5" t="str">
-        <f>VLOOKUP(D2,'[1]Raw data'!1:5,5,0)</f>
-        <v>DRILL BIT 10MM X 116 FLUTE LENGTH (T/S)</v>
+      <c r="D5" t="s">
+        <v>166</v>
       </c>
       <c r="E5" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="11"/>
-      <c r="B6" s="11"/>
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
       <c r="C6" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="D6" t="str">
-        <f>VLOOKUP(D2,'[1]Raw data'!1:6,6,0)</f>
-        <v>EN</v>
+      <c r="D6" t="s">
+        <v>167</v>
       </c>
       <c r="E6" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="11"/>
-      <c r="B7" s="11"/>
+      <c r="A7" s="13"/>
+      <c r="B7" s="13"/>
       <c r="C7" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D7" t="str">
-        <f>VLOOKUP(D2,'[1]Raw data'!1:7,7,0)</f>
-        <v>EA</v>
+      <c r="D7" t="s">
+        <v>168</v>
       </c>
       <c r="E7" t="s">
         <v>99</v>
@@ -1774,24 +1200,23 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="11"/>
-      <c r="B8" s="12" t="s">
+      <c r="A8" s="13"/>
+      <c r="B8" s="14" t="s">
         <v>106</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="D8" t="str">
-        <f>D2</f>
-        <v>CONGEDB0032</v>
+      <c r="D8" t="s">
+        <v>114</v>
       </c>
       <c r="E8" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="11"/>
-      <c r="B9" s="11"/>
+      <c r="A9" s="13"/>
+      <c r="B9" s="13"/>
       <c r="C9" s="4" t="s">
         <v>104</v>
       </c>
@@ -1800,15 +1225,14 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" s="11"/>
-      <c r="B10" s="12" t="s">
+      <c r="A10" s="13"/>
+      <c r="B10" s="14" t="s">
         <v>103</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>102</v>
       </c>
       <c r="D10">
-        <f>VLOOKUP(D2,'[1]Raw data'!1:11,11,0)</f>
         <v>0</v>
       </c>
       <c r="E10" t="s">
@@ -1819,13 +1243,12 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" s="11"/>
-      <c r="B11" s="11"/>
+      <c r="A11" s="13"/>
+      <c r="B11" s="13"/>
       <c r="C11" s="1" t="s">
         <v>101</v>
       </c>
       <c r="D11">
-        <f>VLOOKUP(D2,'[1]Raw data'!1:11,11,0)</f>
         <v>0</v>
       </c>
       <c r="E11" t="s">
@@ -1836,13 +1259,12 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="11"/>
-      <c r="B12" s="11"/>
+      <c r="A12" s="13"/>
+      <c r="B12" s="13"/>
       <c r="C12" s="1" t="s">
         <v>100</v>
       </c>
       <c r="D12">
-        <f>VLOOKUP(D2,'[1]Raw data'!1:10,10,0)</f>
         <v>0</v>
       </c>
       <c r="E12" t="s">
@@ -1853,8 +1275,8 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" s="11"/>
-      <c r="B13" s="12" t="s">
+      <c r="A13" s="13"/>
+      <c r="B13" s="14" t="s">
         <v>98</v>
       </c>
       <c r="C13" s="4" t="s">
@@ -1868,22 +1290,22 @@
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" s="11"/>
-      <c r="B14" s="11"/>
+      <c r="A14" s="13"/>
+      <c r="B14" s="13"/>
       <c r="C14" s="4" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" s="11"/>
-      <c r="B15" s="11"/>
+      <c r="A15" s="13"/>
+      <c r="B15" s="13"/>
       <c r="C15" s="4" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="11"/>
-      <c r="B16" s="12" t="s">
+      <c r="A16" s="13"/>
+      <c r="B16" s="14" t="s">
         <v>5</v>
       </c>
       <c r="C16" s="4" t="s">
@@ -1897,8 +1319,8 @@
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="11"/>
-      <c r="B17" s="11"/>
+      <c r="A17" s="13"/>
+      <c r="B17" s="13"/>
       <c r="C17" s="4" t="s">
         <v>26</v>
       </c>
@@ -1910,8 +1332,8 @@
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A18" s="11"/>
-      <c r="B18" s="11"/>
+      <c r="A18" s="13"/>
+      <c r="B18" s="13"/>
       <c r="C18" s="4" t="s">
         <v>29</v>
       </c>
@@ -1923,8 +1345,8 @@
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A19" s="11"/>
-      <c r="B19" s="11"/>
+      <c r="A19" s="13"/>
+      <c r="B19" s="13"/>
       <c r="C19" s="4" t="s">
         <v>28</v>
       </c>
@@ -1936,23 +1358,22 @@
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="14" t="s">
         <v>20</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D20" t="str">
-        <f>D2</f>
-        <v>CONGEDB0032</v>
+      <c r="D20" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="11"/>
-      <c r="B21" s="11"/>
+      <c r="A21" s="13"/>
+      <c r="B21" s="13"/>
       <c r="C21" s="1" t="s">
         <v>93</v>
       </c>
@@ -1961,8 +1382,8 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="11"/>
-      <c r="B22" s="11"/>
+      <c r="A22" s="13"/>
+      <c r="B22" s="13"/>
       <c r="C22" s="4" t="s">
         <v>91</v>
       </c>
@@ -1975,7 +1396,7 @@
       <c r="F22" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="G22" s="14" t="s">
+      <c r="G22" s="11" t="s">
         <v>126</v>
       </c>
       <c r="H22" t="s">
@@ -1983,7 +1404,7 @@
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="11"/>
+      <c r="A23" s="13"/>
       <c r="B23" s="2" t="s">
         <v>89</v>
       </c>
@@ -2010,23 +1431,22 @@
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A25" s="10" t="s">
+      <c r="A25" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="B25" s="14" t="s">
         <v>20</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D25" t="str">
-        <f>D2</f>
-        <v>CONGEDB0032</v>
+      <c r="D25" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A26" s="11"/>
-      <c r="B26" s="11"/>
+      <c r="A26" s="13"/>
+      <c r="B26" s="13"/>
       <c r="C26" s="4" t="s">
         <v>85</v>
       </c>
@@ -2041,8 +1461,8 @@
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A27" s="11"/>
-      <c r="B27" s="12" t="s">
+      <c r="A27" s="13"/>
+      <c r="B27" s="14" t="s">
         <v>83</v>
       </c>
       <c r="C27" s="4" t="s">
@@ -2059,8 +1479,8 @@
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A28" s="11"/>
-      <c r="B28" s="11"/>
+      <c r="A28" s="13"/>
+      <c r="B28" s="13"/>
       <c r="C28" s="4" t="s">
         <v>79</v>
       </c>
@@ -2075,8 +1495,8 @@
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A29" s="11"/>
-      <c r="B29" s="11"/>
+      <c r="A29" s="13"/>
+      <c r="B29" s="13"/>
       <c r="C29" s="4" t="s">
         <v>78</v>
       </c>
@@ -2091,8 +1511,8 @@
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A30" s="11"/>
-      <c r="B30" s="11"/>
+      <c r="A30" s="13"/>
+      <c r="B30" s="13"/>
       <c r="C30" s="4" t="s">
         <v>75</v>
       </c>
@@ -2107,8 +1527,8 @@
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A31" s="11"/>
-      <c r="B31" s="11"/>
+      <c r="A31" s="13"/>
+      <c r="B31" s="13"/>
       <c r="C31" s="4" t="s">
         <v>74</v>
       </c>
@@ -2123,8 +1543,8 @@
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" s="11"/>
-      <c r="B32" s="11"/>
+      <c r="A32" s="13"/>
+      <c r="B32" s="13"/>
       <c r="C32" s="4" t="s">
         <v>71</v>
       </c>
@@ -2139,8 +1559,8 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A33" s="11"/>
-      <c r="B33" s="11"/>
+      <c r="A33" s="13"/>
+      <c r="B33" s="13"/>
       <c r="C33" s="4" t="s">
         <v>70</v>
       </c>
@@ -2155,8 +1575,8 @@
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A34" s="11"/>
-      <c r="B34" s="11"/>
+      <c r="A34" s="13"/>
+      <c r="B34" s="13"/>
       <c r="C34" s="4" t="s">
         <v>67</v>
       </c>
@@ -2171,8 +1591,8 @@
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A35" s="11"/>
-      <c r="B35" s="11"/>
+      <c r="A35" s="13"/>
+      <c r="B35" s="13"/>
       <c r="C35" s="4" t="s">
         <v>64</v>
       </c>
@@ -2187,8 +1607,8 @@
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A36" s="11"/>
-      <c r="B36" s="11"/>
+      <c r="A36" s="13"/>
+      <c r="B36" s="13"/>
       <c r="C36" s="4" t="s">
         <v>61</v>
       </c>
@@ -2203,8 +1623,8 @@
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A37" s="11"/>
-      <c r="B37" s="11"/>
+      <c r="A37" s="13"/>
+      <c r="B37" s="13"/>
       <c r="C37" s="4" t="s">
         <v>60</v>
       </c>
@@ -2219,8 +1639,8 @@
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A38" s="11"/>
-      <c r="B38" s="11"/>
+      <c r="A38" s="13"/>
+      <c r="B38" s="13"/>
       <c r="C38" s="4" t="s">
         <v>57</v>
       </c>
@@ -2235,23 +1655,22 @@
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A39" s="10" t="s">
+      <c r="A39" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="B39" s="12" t="s">
+      <c r="B39" s="14" t="s">
         <v>20</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D39" t="str">
-        <f>D2</f>
-        <v>CONGEDB0032</v>
+      <c r="D39" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A40" s="11"/>
-      <c r="B40" s="11"/>
+      <c r="A40" s="13"/>
+      <c r="B40" s="13"/>
       <c r="C40" s="4" t="s">
         <v>23</v>
       </c>
@@ -2266,8 +1685,8 @@
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A41" s="11"/>
-      <c r="B41" s="12" t="s">
+      <c r="A41" s="13"/>
+      <c r="B41" s="14" t="s">
         <v>52</v>
       </c>
       <c r="C41" s="1" t="s">
@@ -2281,8 +1700,8 @@
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A42" s="11"/>
-      <c r="B42" s="12"/>
+      <c r="A42" s="13"/>
+      <c r="B42" s="14"/>
       <c r="C42" s="1" t="s">
         <v>153</v>
       </c>
@@ -2294,8 +1713,8 @@
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A43" s="11"/>
-      <c r="B43" s="11"/>
+      <c r="A43" s="13"/>
+      <c r="B43" s="13"/>
       <c r="C43" s="1" t="s">
         <v>49</v>
       </c>
@@ -2310,8 +1729,8 @@
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A44" s="11"/>
-      <c r="B44" s="12" t="s">
+      <c r="A44" s="13"/>
+      <c r="B44" s="14" t="s">
         <v>46</v>
       </c>
       <c r="C44" s="1" t="s">
@@ -2331,8 +1750,8 @@
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A45" s="11"/>
-      <c r="B45" s="11"/>
+      <c r="A45" s="13"/>
+      <c r="B45" s="13"/>
       <c r="C45" s="1" t="s">
         <v>44</v>
       </c>
@@ -2344,8 +1763,8 @@
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A46" s="11"/>
-      <c r="B46" s="11"/>
+      <c r="A46" s="13"/>
+      <c r="B46" s="13"/>
       <c r="C46" s="1" t="s">
         <v>43</v>
       </c>
@@ -2357,7 +1776,7 @@
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A47" s="11"/>
+      <c r="A47" s="13"/>
       <c r="C47" s="1" t="s">
         <v>41</v>
       </c>
@@ -2367,7 +1786,7 @@
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A48" s="11"/>
+      <c r="A48" s="13"/>
       <c r="B48" s="2" t="s">
         <v>39</v>
       </c>
@@ -2382,7 +1801,7 @@
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A49" s="11"/>
+      <c r="A49" s="13"/>
       <c r="B49" s="2"/>
       <c r="C49" s="1" t="s">
         <v>155</v>
@@ -2395,7 +1814,7 @@
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A50" s="11"/>
+      <c r="A50" s="13"/>
       <c r="B50" s="2"/>
       <c r="C50" s="1" t="s">
         <v>157</v>
@@ -2405,7 +1824,7 @@
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A51" s="11"/>
+      <c r="A51" s="13"/>
       <c r="B51" s="2"/>
       <c r="C51" s="1" t="s">
         <v>158</v>
@@ -2421,7 +1840,7 @@
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A52" s="11"/>
+      <c r="A52" s="13"/>
       <c r="B52" s="2" t="s">
         <v>36</v>
       </c>
@@ -2436,7 +1855,7 @@
       </c>
     </row>
     <row r="53" spans="1:9" ht="64" x14ac:dyDescent="0.2">
-      <c r="A53" s="11"/>
+      <c r="A53" s="13"/>
       <c r="B53" s="2" t="s">
         <v>33</v>
       </c>
@@ -2454,8 +1873,8 @@
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A54" s="11"/>
-      <c r="B54" s="12" t="s">
+      <c r="A54" s="13"/>
+      <c r="B54" s="14" t="s">
         <v>5</v>
       </c>
       <c r="C54" s="1" t="s">
@@ -2469,8 +1888,8 @@
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A55" s="11"/>
-      <c r="B55" s="12"/>
+      <c r="A55" s="13"/>
+      <c r="B55" s="14"/>
       <c r="C55" s="1" t="s">
         <v>162</v>
       </c>
@@ -2479,8 +1898,8 @@
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A56" s="11"/>
-      <c r="B56" s="11"/>
+      <c r="A56" s="13"/>
+      <c r="B56" s="13"/>
       <c r="C56" s="1" t="s">
         <v>28</v>
       </c>
@@ -2492,8 +1911,8 @@
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A57" s="11"/>
-      <c r="B57" s="11"/>
+      <c r="A57" s="13"/>
+      <c r="B57" s="13"/>
       <c r="C57" s="1" t="s">
         <v>27</v>
       </c>
@@ -2505,8 +1924,8 @@
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A58" s="11"/>
-      <c r="B58" s="11"/>
+      <c r="A58" s="13"/>
+      <c r="B58" s="13"/>
       <c r="C58" s="1" t="s">
         <v>26</v>
       </c>
@@ -2518,10 +1937,10 @@
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A59" s="10" t="s">
+      <c r="A59" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B59" s="12" t="s">
+      <c r="B59" s="14" t="s">
         <v>20</v>
       </c>
       <c r="C59" s="3" t="s">
@@ -2532,8 +1951,8 @@
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A60" s="11"/>
-      <c r="B60" s="11"/>
+      <c r="A60" s="13"/>
+      <c r="B60" s="13"/>
       <c r="C60" s="4" t="s">
         <v>23</v>
       </c>
@@ -2542,8 +1961,8 @@
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A61" s="11"/>
-      <c r="B61" s="11"/>
+      <c r="A61" s="13"/>
+      <c r="B61" s="13"/>
       <c r="C61" s="1" t="s">
         <v>22</v>
       </c>
@@ -2561,23 +1980,22 @@
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A62" s="10" t="s">
+      <c r="A62" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B62" s="12" t="s">
+      <c r="B62" s="14" t="s">
         <v>20</v>
       </c>
       <c r="C62" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D62" t="str">
-        <f>D20</f>
-        <v>CONGEDB0032</v>
+      <c r="D62" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A63" s="11"/>
-      <c r="B63" s="11"/>
+      <c r="A63" s="13"/>
+      <c r="B63" s="13"/>
       <c r="C63" s="1" t="s">
         <v>18</v>
       </c>
@@ -2592,8 +2010,8 @@
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A64" s="11"/>
-      <c r="B64" s="12" t="s">
+      <c r="A64" s="13"/>
+      <c r="B64" s="14" t="s">
         <v>16</v>
       </c>
       <c r="C64" s="1" t="s">
@@ -2610,8 +2028,8 @@
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A65" s="11"/>
-      <c r="B65" s="11"/>
+      <c r="A65" s="13"/>
+      <c r="B65" s="13"/>
       <c r="C65" s="1" t="s">
         <v>13</v>
       </c>
@@ -2626,8 +2044,8 @@
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A66" s="11"/>
-      <c r="B66" s="12" t="s">
+      <c r="A66" s="13"/>
+      <c r="B66" s="14" t="s">
         <v>12</v>
       </c>
       <c r="C66" s="1" t="s">
@@ -2641,8 +2059,8 @@
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A67" s="11"/>
-      <c r="B67" s="11"/>
+      <c r="A67" s="13"/>
+      <c r="B67" s="13"/>
       <c r="C67" s="1" t="s">
         <v>8</v>
       </c>
@@ -2654,8 +2072,8 @@
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A68" s="11"/>
-      <c r="B68" s="12" t="s">
+      <c r="A68" s="13"/>
+      <c r="B68" s="14" t="s">
         <v>5</v>
       </c>
       <c r="C68" s="1" t="s">
@@ -2672,8 +2090,8 @@
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A69" s="11"/>
-      <c r="B69" s="11"/>
+      <c r="A69" s="13"/>
+      <c r="B69" s="13"/>
       <c r="C69" s="1" t="s">
         <v>3</v>
       </c>
@@ -2689,22 +2107,6 @@
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="A2:A19"/>
-    <mergeCell ref="B3:B7"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="B16:B19"/>
-    <mergeCell ref="A20:A23"/>
-    <mergeCell ref="B20:B22"/>
-    <mergeCell ref="A25:A38"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="B27:B38"/>
-    <mergeCell ref="A39:A58"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="B44:B46"/>
-    <mergeCell ref="B54:B58"/>
     <mergeCell ref="A59:A61"/>
     <mergeCell ref="B59:B61"/>
     <mergeCell ref="A62:A69"/>
@@ -2712,6 +2114,22 @@
     <mergeCell ref="B64:B65"/>
     <mergeCell ref="B66:B67"/>
     <mergeCell ref="B68:B69"/>
+    <mergeCell ref="A39:A58"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="B54:B58"/>
+    <mergeCell ref="A20:A23"/>
+    <mergeCell ref="B20:B22"/>
+    <mergeCell ref="A25:A38"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="B27:B38"/>
+    <mergeCell ref="A2:A19"/>
+    <mergeCell ref="B3:B7"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="B16:B19"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="G3" r:id="rId1" xr:uid="{B7C850E2-54B8-A241-9481-8B7E19688D42}"/>

</xml_diff>